<commit_message>
Apply approved grocery categories and add chilled fresh section
</commit_message>
<xml_diff>
--- a/public/images/items/ingredienten_categorieen.xlsx
+++ b/public/images/items/ingredienten_categorieen.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorieën" sheetId="1" r:id="Rfd94c4e875fc401f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ingrediënten" sheetId="2" r:id="R36f30d6091654936"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synoniemen" sheetId="3" r:id="Rca14c7ce7e6c4f32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorieën" sheetId="1" r:id="R6187029827dd4198"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ingrediënten" sheetId="2" r:id="Rc013a4ccea0d41c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synoniemen" sheetId="3" r:id="R0ee6f4654a1a4665"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -308,66 +308,71 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>Brood</x:v>
+        <x:v>Gekoeld &amp; Vers</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Beleg</x:v>
+        <x:v>Brood</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>Droogwaren &amp; Bakproducten</x:v>
+        <x:v>Beleg</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>Conserven, Sauzen, Olie &amp; Kruiden</x:v>
+        <x:v>Droogwaren &amp; Bakproducten</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>Zoute Snacks</x:v>
+        <x:v>Conserven, Sauzen, Olie &amp; Kruiden</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>Snoep &amp; Chocolade</x:v>
+        <x:v>Zoute Snacks</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>Warme Dranken</x:v>
+        <x:v>Snoep &amp; Chocolade</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>Koude Dranken</x:v>
+        <x:v>Warme Dranken</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>Diepvries</x:v>
+        <x:v>Koude Dranken</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>Huishouden &amp; Schoonmaak</x:v>
+        <x:v>Diepvries</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>Persoonlijke Verzorging</x:v>
+        <x:v>Huishouden &amp; Schoonmaak</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>Dierenvoeding</x:v>
+        <x:v>Persoonlijke Verzorging</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
+        <x:v>Dierenvoeding</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
         <x:v>Overig</x:v>
       </x:c>
     </x:row>
@@ -632,7 +637,7 @@
         <x:v>bladerdeeg</x:v>
       </x:c>
       <x:c r="B32" t="str">
-        <x:v>Zuivel, Kaas &amp; Eieren</x:v>
+        <x:v>Gekoeld &amp; Vers</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -1160,7 +1165,7 @@
         <x:v>gevulde pasta</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Droogwaren &amp; Bakproducten</x:v>
+        <x:v>Gekoeld &amp; Vers</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -2688,7 +2693,7 @@
         <x:v>verse gist</x:v>
       </x:c>
       <x:c r="B289" t="str">
-        <x:v>Droogwaren &amp; Bakproducten</x:v>
+        <x:v>Gekoeld &amp; Vers</x:v>
       </x:c>
     </x:row>
     <x:row r="290">
@@ -3040,7 +3045,7 @@
         <x:v>vol-au-vent_koekje</x:v>
       </x:c>
       <x:c r="B333" t="str">
-        <x:v>Diepvries</x:v>
+        <x:v>Brood</x:v>
       </x:c>
     </x:row>
     <x:row r="334">
@@ -3048,7 +3053,7 @@
         <x:v>vol-au-vent_voorgemaakt</x:v>
       </x:c>
       <x:c r="B334" t="str">
-        <x:v>Diepvries</x:v>
+        <x:v>Vlees &amp; Charcuterie</x:v>
       </x:c>
     </x:row>
     <x:row r="335">
@@ -3065,6 +3070,414 @@
       </x:c>
       <x:c r="B336" t="str">
         <x:v>Vlees &amp; Charcuterie</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="337">
+      <x:c r="A337" t="str">
+        <x:v>blik tomaten</x:v>
+      </x:c>
+      <x:c r="B337" t="str">
+        <x:v>Conserven, Sauzen, Olie &amp; Kruiden</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="338">
+      <x:c r="A338" t="str">
+        <x:v>rode curry pasta</x:v>
+      </x:c>
+      <x:c r="B338" t="str">
+        <x:v>Conserven, Sauzen, Olie &amp; Kruiden</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="339">
+      <x:c r="A339" t="str">
+        <x:v>ajuinpoeder</x:v>
+      </x:c>
+      <x:c r="B339" t="str">
+        <x:v>Conserven, Sauzen, Olie &amp; Kruiden</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="340">
+      <x:c r="A340" t="str">
+        <x:v>look granulaat</x:v>
+      </x:c>
+      <x:c r="B340" t="str">
+        <x:v>Conserven, Sauzen, Olie &amp; Kruiden</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="341">
+      <x:c r="A341" t="str">
+        <x:v>gefrituurde ajuin</x:v>
+      </x:c>
+      <x:c r="B341" t="str">
+        <x:v>Conserven, Sauzen, Olie &amp; Kruiden</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="342">
+      <x:c r="A342" t="str">
+        <x:v>pizzasaus</x:v>
+      </x:c>
+      <x:c r="B342" t="str">
+        <x:v>Conserven, Sauzen, Olie &amp; Kruiden</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="343">
+      <x:c r="A343" t="str">
+        <x:v>tomatensaus</x:v>
+      </x:c>
+      <x:c r="B343" t="str">
+        <x:v>Conserven, Sauzen, Olie &amp; Kruiden</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="344">
+      <x:c r="A344" t="str">
+        <x:v>00-bloem</x:v>
+      </x:c>
+      <x:c r="B344" t="str">
+        <x:v>Droogwaren &amp; Bakproducten</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="345">
+      <x:c r="A345" t="str">
+        <x:v>droge gist</x:v>
+      </x:c>
+      <x:c r="B345" t="str">
+        <x:v>Droogwaren &amp; Bakproducten</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="346">
+      <x:c r="A346" t="str">
+        <x:v>pannekoekenmix</x:v>
+      </x:c>
+      <x:c r="B346" t="str">
+        <x:v>Droogwaren &amp; Bakproducten</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="347">
+      <x:c r="A347" t="str">
+        <x:v>zelfrijzend bakmeel</x:v>
+      </x:c>
+      <x:c r="B347" t="str">
+        <x:v>Droogwaren &amp; Bakproducten</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="348">
+      <x:c r="A348" t="str">
+        <x:v>zusto zoetstof</x:v>
+      </x:c>
+      <x:c r="B348" t="str">
+        <x:v>Droogwaren &amp; Bakproducten</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="349">
+      <x:c r="A349" t="str">
+        <x:v>gehakte walnoten</x:v>
+      </x:c>
+      <x:c r="B349" t="str">
+        <x:v>Droogwaren &amp; Bakproducten</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="350">
+      <x:c r="A350" t="str">
+        <x:v>boursin</x:v>
+      </x:c>
+      <x:c r="B350" t="str">
+        <x:v>Zuivel, Kaas &amp; Eieren</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="351">
+      <x:c r="A351" t="str">
+        <x:v>parmezaan</x:v>
+      </x:c>
+      <x:c r="B351" t="str">
+        <x:v>Zuivel, Kaas &amp; Eieren</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="352">
+      <x:c r="A352" t="str">
+        <x:v>tete de moine</x:v>
+      </x:c>
+      <x:c r="B352" t="str">
+        <x:v>Zuivel, Kaas &amp; Eieren</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="353">
+      <x:c r="A353" t="str">
+        <x:v>aardpeer</x:v>
+      </x:c>
+      <x:c r="B353" t="str">
+        <x:v>Groenten &amp; Fruit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="354">
+      <x:c r="A354" t="str">
+        <x:v>kiwis</x:v>
+      </x:c>
+      <x:c r="B354" t="str">
+        <x:v>Groenten &amp; Fruit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="355">
+      <x:c r="A355" t="str">
+        <x:v>mango</x:v>
+      </x:c>
+      <x:c r="B355" t="str">
+        <x:v>Groenten &amp; Fruit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="356">
+      <x:c r="A356" t="str">
+        <x:v>zespri gold</x:v>
+      </x:c>
+      <x:c r="B356" t="str">
+        <x:v>Groenten &amp; Fruit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="357">
+      <x:c r="A357" t="str">
+        <x:v>verse dille</x:v>
+      </x:c>
+      <x:c r="B357" t="str">
+        <x:v>Groenten &amp; Fruit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="358">
+      <x:c r="A358" t="str">
+        <x:v>af te bakken broodje</x:v>
+      </x:c>
+      <x:c r="B358" t="str">
+        <x:v>Brood</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="359">
+      <x:c r="A359" t="str">
+        <x:v>piccolo broodje</x:v>
+      </x:c>
+      <x:c r="B359" t="str">
+        <x:v>Brood</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="360">
+      <x:c r="A360" t="str">
+        <x:v>roze red bull</x:v>
+      </x:c>
+      <x:c r="B360" t="str">
+        <x:v>Koude Dranken</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="361">
+      <x:c r="A361" t="str">
+        <x:v>witte red bull</x:v>
+      </x:c>
+      <x:c r="B361" t="str">
+        <x:v>Koude Dranken</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="362">
+      <x:c r="A362" t="str">
+        <x:v>kombucha</x:v>
+      </x:c>
+      <x:c r="B362" t="str">
+        <x:v>Koude Dranken</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="363">
+      <x:c r="A363" t="str">
+        <x:v>kippenboutjes</x:v>
+      </x:c>
+      <x:c r="B363" t="str">
+        <x:v>Vlees &amp; Charcuterie</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="364">
+      <x:c r="A364" t="str">
+        <x:v>schnitzels</x:v>
+      </x:c>
+      <x:c r="B364" t="str">
+        <x:v>Vlees &amp; Charcuterie</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="365">
+      <x:c r="A365" t="str">
+        <x:v>plastic wrap</x:v>
+      </x:c>
+      <x:c r="B365" t="str">
+        <x:v>Huishouden &amp; Schoonmaak</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="366">
+      <x:c r="A366" t="str">
+        <x:v>oorstokjes</x:v>
+      </x:c>
+      <x:c r="B366" t="str">
+        <x:v>Persoonlijke Verzorging</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="367">
+      <x:c r="A367" t="str">
+        <x:v>chocoladeparels</x:v>
+      </x:c>
+      <x:c r="B367" t="str">
+        <x:v>Snoep &amp; Chocolade</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="368">
+      <x:c r="A368" t="str">
+        <x:v>paaseieren noe</x:v>
+      </x:c>
+      <x:c r="B368" t="str">
+        <x:v>Snoep &amp; Chocolade</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="369">
+      <x:c r="A369" t="str">
+        <x:v>scampi look chloe</x:v>
+      </x:c>
+      <x:c r="B369" t="str">
+        <x:v>Vis &amp; Zeevruchten</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="370">
+      <x:c r="A370" t="str">
+        <x:v>hot dogs</x:v>
+      </x:c>
+      <x:c r="B370" t="str">
+        <x:v>Conserven, Sauzen, Olie &amp; Kruiden</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="371">
+      <x:c r="A371" t="str">
+        <x:v>knijpzakjes appel/banaan chloe</x:v>
+      </x:c>
+      <x:c r="B371" t="str">
+        <x:v>Conserven, Sauzen, Olie &amp; Kruiden</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="372">
+      <x:c r="A372" t="str">
+        <x:v>ovenhapjes</x:v>
+      </x:c>
+      <x:c r="B372" t="str">
+        <x:v>Diepvries</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="373">
+      <x:c r="A373" t="str">
+        <x:v>fish sticks</x:v>
+      </x:c>
+      <x:c r="B373" t="str">
+        <x:v>Diepvries</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="374">
+      <x:c r="A374" t="str">
+        <x:v>groentjes igloo</x:v>
+      </x:c>
+      <x:c r="B374" t="str">
+        <x:v>Diepvries</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="375">
+      <x:c r="A375" t="str">
+        <x:v>iglo bowls noodles kip</x:v>
+      </x:c>
+      <x:c r="B375" t="str">
+        <x:v>Diepvries</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="376">
+      <x:c r="A376" t="str">
+        <x:v>wortelen (diepvries)</x:v>
+      </x:c>
+      <x:c r="B376" t="str">
+        <x:v>Diepvries</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="377">
+      <x:c r="A377" t="str">
+        <x:v>verse pasta</x:v>
+      </x:c>
+      <x:c r="B377" t="str">
+        <x:v>Gekoeld &amp; Vers</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="378">
+      <x:c r="A378" t="str">
+        <x:v>krabsla</x:v>
+      </x:c>
+      <x:c r="B378" t="str">
+        <x:v>Beleg</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="379">
+      <x:c r="A379" t="str">
+        <x:v>verse basilicum</x:v>
+      </x:c>
+      <x:c r="B379" t="str">
+        <x:v>Groenten &amp; Fruit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="380">
+      <x:c r="A380" t="str">
+        <x:v>gedroogde basilicum</x:v>
+      </x:c>
+      <x:c r="B380" t="str">
+        <x:v>Conserven, Sauzen, Olie &amp; Kruiden</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="381">
+      <x:c r="A381" t="str">
+        <x:v>verse tijm</x:v>
+      </x:c>
+      <x:c r="B381" t="str">
+        <x:v>Groenten &amp; Fruit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="382">
+      <x:c r="A382" t="str">
+        <x:v>gedroogde tijm</x:v>
+      </x:c>
+      <x:c r="B382" t="str">
+        <x:v>Conserven, Sauzen, Olie &amp; Kruiden</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="383">
+      <x:c r="A383" t="str">
+        <x:v>verse koriander</x:v>
+      </x:c>
+      <x:c r="B383" t="str">
+        <x:v>Groenten &amp; Fruit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="384">
+      <x:c r="A384" t="str">
+        <x:v>gedroogde koriander</x:v>
+      </x:c>
+      <x:c r="B384" t="str">
+        <x:v>Conserven, Sauzen, Olie &amp; Kruiden</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="385">
+      <x:c r="A385" t="str">
+        <x:v>verse peterselie</x:v>
+      </x:c>
+      <x:c r="B385" t="str">
+        <x:v>Groenten &amp; Fruit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="386">
+      <x:c r="A386" t="str">
+        <x:v>gedroogde peterselie</x:v>
+      </x:c>
+      <x:c r="B386" t="str">
+        <x:v>Conserven, Sauzen, Olie &amp; Kruiden</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="387">
+      <x:c r="A387" t="str">
+        <x:v>gedroogde dille</x:v>
+      </x:c>
+      <x:c r="B387" t="str">
+        <x:v>Conserven, Sauzen, Olie &amp; Kruiden</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>